<commit_message>
Added LPG OI and mapping for the alerts
</commit_message>
<xml_diff>
--- a/orchestrator/masters/PerformanceIndex_Rules.xlsx
+++ b/orchestrator/masters/PerformanceIndex_Rules.xlsx
@@ -1,49 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10119"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/venugopalnaidu/Documents/HPCL/OI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac_1/PycharmProjects/Cloud/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD51BDAA-BC05-9441-8F17-CAC5FB6B45C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1BF56D-83D4-B448-846B-56B1CC144C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="16020" xr2:uid="{52EB7FBB-DAEB-0D47-9698-3EE15E213270}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAS" sheetId="1" r:id="rId1"/>
+    <sheet name="LPG" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
   <si>
     <t>BU</t>
   </si>
   <si>
+    <t>AlertSection</t>
+  </si>
+  <si>
+    <t>DeviceCategory</t>
+  </si>
+  <si>
     <t>Weightage</t>
   </si>
   <si>
+    <t>Enabled</t>
+  </si>
+  <si>
     <t>TAS</t>
   </si>
   <si>
@@ -53,9 +47,6 @@
     <t>Safety</t>
   </si>
   <si>
-    <t>DeviceCategory</t>
-  </si>
-  <si>
     <t>FE&amp;Jockey</t>
   </si>
   <si>
@@ -65,9 +56,6 @@
     <t>FoamQty</t>
   </si>
   <si>
-    <t>Enabled</t>
-  </si>
-  <si>
     <t>PT</t>
   </si>
   <si>
@@ -83,25 +71,88 @@
     <t>EMLock</t>
   </si>
   <si>
-    <t>AlertSection</t>
+    <t>LPG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check Scale alerts </t>
+  </si>
+  <si>
+    <t>Check Scale Rejection</t>
+  </si>
+  <si>
+    <t>&lt;/=3 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valve leak alerts </t>
+  </si>
+  <si>
+    <t>&gt;8%</t>
+  </si>
+  <si>
+    <t>&gt;3 to 8 %</t>
+  </si>
+  <si>
+    <t>0 to 100%</t>
+  </si>
+  <si>
+    <t>&gt;6%</t>
+  </si>
+  <si>
+    <t>&gt;3 to 6 %</t>
+  </si>
+  <si>
+    <t>&lt;/=6 %</t>
+  </si>
+  <si>
+    <t>Valve Leakage Rejection</t>
+  </si>
+  <si>
+    <t>&gt;12%</t>
+  </si>
+  <si>
+    <t>O-Ring Leakage Rejection</t>
+  </si>
+  <si>
+    <t>&gt;6 to 12 %</t>
+  </si>
+  <si>
+    <t>Rejections</t>
+  </si>
+  <si>
+    <t>Score</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mmm"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -132,9 +183,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -195,7 +261,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -228,26 +294,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -280,23 +329,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -459,18 +491,13 @@
     </a:lnDef>
   </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D65289C-8F83-B24F-AA10-1791750CEE08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.5" customWidth="1"/>
     <col min="3" max="3" width="23.1640625" customWidth="1"/>
@@ -482,27 +509,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D2">
         <v>15</v>
@@ -513,13 +540,13 @@
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D3">
         <v>20</v>
@@ -530,13 +557,13 @@
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>10</v>
@@ -547,13 +574,13 @@
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -564,13 +591,13 @@
     </row>
     <row r="6" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6">
         <v>5</v>
@@ -581,13 +608,13 @@
     </row>
     <row r="7" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -598,10 +625,10 @@
     </row>
     <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -612,10 +639,10 @@
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>10</v>
@@ -626,10 +653,10 @@
     </row>
     <row r="10" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10">
         <v>15</v>
@@ -640,10 +667,10 @@
     </row>
     <row r="11" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>5</v>
@@ -653,6 +680,198 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776A0F6A-0986-F548-BBB9-BD8DA35647E4}">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="6">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="6">
+        <v>35</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="6">
+        <v>35</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G10" s="5"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="G2:G4"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="G5:G7"/>
+    <mergeCell ref="B8:B10"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated the category mapping and rules sheet
</commit_message>
<xml_diff>
--- a/orchestrator/masters/PerformanceIndex_Rules.xlsx
+++ b/orchestrator/masters/PerformanceIndex_Rules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac_1/PycharmProjects/Cloud/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1BF56D-83D4-B448-846B-56B1CC144C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACF8DAA-86CB-6B45-9AA3-B1403D99DDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="30">
   <si>
     <t>BU</t>
   </si>
@@ -77,9 +77,6 @@
     <t xml:space="preserve">Check Scale alerts </t>
   </si>
   <si>
-    <t>Check Scale Rejection</t>
-  </si>
-  <si>
     <t>&lt;/=3 %</t>
   </si>
   <si>
@@ -104,13 +101,7 @@
     <t>&lt;/=6 %</t>
   </si>
   <si>
-    <t>Valve Leakage Rejection</t>
-  </si>
-  <si>
     <t>&gt;12%</t>
-  </si>
-  <si>
-    <t>O-Ring Leakage Rejection</t>
   </si>
   <si>
     <t>&gt;6 to 12 %</t>
@@ -689,6 +680,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776A0F6A-0986-F548-BBB9-BD8DA35647E4}">
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -704,10 +703,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
@@ -718,16 +717,16 @@
         <v>16</v>
       </c>
       <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>18</v>
       </c>
       <c r="D2" s="6">
         <v>30</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F2" s="3">
         <v>1</v>
@@ -742,7 +741,7 @@
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F3" s="3">
         <v>0</v>
@@ -755,26 +754,26 @@
       <c r="C4" s="5"/>
       <c r="D4" s="6"/>
       <c r="E4" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="G4" s="5"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="D5" s="6">
         <v>35</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -789,7 +788,7 @@
       <c r="C6" s="5"/>
       <c r="D6" s="6"/>
       <c r="E6" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F6" s="3">
         <v>0</v>
@@ -802,26 +801,26 @@
       <c r="C7" s="5"/>
       <c r="D7" s="6"/>
       <c r="E7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G7" s="5"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="D8" s="6">
         <v>35</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F8" s="3">
         <v>1</v>
@@ -836,7 +835,7 @@
       <c r="C9" s="5"/>
       <c r="D9" s="6"/>
       <c r="E9" s="2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F9" s="3">
         <v>0</v>
@@ -849,10 +848,10 @@
       <c r="C10" s="5"/>
       <c r="D10" s="6"/>
       <c r="E10" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G10" s="5"/>
     </row>

</xml_diff>

<commit_message>
Updated Tas OI, rules sheet, category mapping,
</commit_message>
<xml_diff>
--- a/orchestrator/masters/PerformanceIndex_Rules.xlsx
+++ b/orchestrator/masters/PerformanceIndex_Rules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac_1/PycharmProjects/Cloud/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACF8DAA-86CB-6B45-9AA3-B1403D99DDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE216B-68BC-1245-AF83-89B1376FA894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="31">
   <si>
     <t>BU</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>Score</t>
+  </si>
+  <si>
+    <t>Gantry</t>
   </si>
 </sst>
 </file>
@@ -120,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mmm"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -140,6 +143,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
@@ -174,9 +183,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -186,7 +196,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -487,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.5" customWidth="1"/>
@@ -587,11 +597,11 @@
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
-        <v>10</v>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -605,7 +615,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -619,13 +629,16 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
       </c>
       <c r="D8">
         <v>5</v>
       </c>
       <c r="E8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -633,10 +646,10 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -647,10 +660,10 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -661,12 +674,26 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11">
         <v>15</v>
       </c>
-      <c r="D11">
-        <v>5</v>
-      </c>
       <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12">
+        <v>5</v>
+      </c>
+      <c r="E12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -713,147 +740,147 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="7">
         <v>30</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="3">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5" t="b">
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="2" t="s">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="4">
         <v>0</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="4" t="s">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5" t="s">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="7">
         <v>35</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="3">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="b">
+      <c r="F5" s="4">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="2" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>0</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="4" t="s">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G7" s="5"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5" t="s">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="7">
         <v>35</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="3">
-        <v>1</v>
-      </c>
-      <c r="G8" s="5" t="b">
+      <c r="F8" s="4">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="2" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F9" s="4">
         <v>0</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="4" t="s">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="5"/>
+      <c r="G10" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>

<commit_message>
Updated TAS and LPG oi code
</commit_message>
<xml_diff>
--- a/orchestrator/masters/PerformanceIndex_Rules.xlsx
+++ b/orchestrator/masters/PerformanceIndex_Rules.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10209"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac_1/PycharmProjects/Cloud/dnc_backend_v2/orchestrator/masters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/venugopalnaidu/PycharmProjects/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE216B-68BC-1245-AF83-89B1376FA894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328EFBEF-641F-1C45-BA4A-98A612F7EAF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32380" yWindow="2580" windowWidth="28800" windowHeight="16520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TAS" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="31">
   <si>
     <t>BU</t>
   </si>
@@ -74,15 +74,9 @@
     <t>LPG</t>
   </si>
   <si>
-    <t xml:space="preserve">Check Scale alerts </t>
-  </si>
-  <si>
     <t>&lt;/=3 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Valve leak alerts </t>
-  </si>
-  <si>
     <t>&gt;8%</t>
   </si>
   <si>
@@ -113,7 +107,13 @@
     <t>Score</t>
   </si>
   <si>
-    <t>Gantry</t>
+    <t>Check Scale Rejection</t>
+  </si>
+  <si>
+    <t>O-Ring Leak Rejection</t>
+  </si>
+  <si>
+    <t>Valve Leak Rejection</t>
   </si>
 </sst>
 </file>
@@ -123,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mmm"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -143,12 +143,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
@@ -183,10 +177,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -196,7 +189,7 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -497,7 +490,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="21" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="17.5" customWidth="1"/>
@@ -597,11 +590,11 @@
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
+      <c r="C6" t="s">
+        <v>10</v>
       </c>
       <c r="D6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -615,7 +608,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7">
         <v>5</v>
@@ -629,16 +622,13 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8">
         <v>5</v>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
@@ -646,10 +636,10 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -660,10 +650,10 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -674,26 +664,12 @@
         <v>5</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D11">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E11" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D12">
-        <v>5</v>
-      </c>
-      <c r="E12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -705,7 +681,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{776A0F6A-0986-F548-BBB9-BD8DA35647E4}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.33203125" bestFit="1" customWidth="1"/>
@@ -730,157 +706,185 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="6">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="7">
+      <c r="F2" s="3">
+        <v>1</v>
+      </c>
+      <c r="G2" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0</v>
+      </c>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="5"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" s="4">
-        <v>1</v>
-      </c>
-      <c r="G2" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="3" t="s">
+      <c r="D5" s="6">
+        <v>35</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="4">
+      <c r="G7" s="5"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="6">
+        <v>35</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="3">
         <v>0</v>
       </c>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="7">
-        <v>35</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="4">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0</v>
-      </c>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="7">
-        <v>35</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="G9" s="5"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="4">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F9" s="4">
-        <v>0</v>
-      </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G10" s="6"/>
+      <c r="F10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="5"/>
+    </row>
+    <row r="11" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11">
+        <v>5</v>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>